<commit_message>
send emails with attachment+ store email results in excel
</commit_message>
<xml_diff>
--- a/test_cases/RamaNamaCerti.xlsx
+++ b/test_cases/RamaNamaCerti.xlsx
@@ -5,22 +5,23 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Email Results" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
     <t xml:space="preserve">emails</t>
   </si>
@@ -37,37 +38,13 @@
     <t xml:space="preserve">shashank</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">14</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">th</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> aug 1996</t>
-    </r>
+    <t xml:space="preserve">14th august 1996</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sheshu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14th december 1998</t>
   </si>
   <si>
     <t xml:space="preserve">h20191030599@hyderabad.bits-pilani.ac.in</t>
@@ -76,37 +53,37 @@
     <t xml:space="preserve">paravasthu</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">th</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> march 1998</t>
-    </r>
+    <t xml:space="preserve">20th march 1998</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hemapkrishna@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6th Feb 1993</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arkvidhatha@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17th november 1997</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Errno 2] No such file or directory: '/home/paravasthu/ghostee/mailSender/test_cases/test_attachments/shashank.jpg'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{'shashank': (553, b'5.1.3 The recipient address &lt;shashank&gt; is not a valid RFC-5321 address. kf10sm2286206pjb.2 - gsmtp')}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sent mail to: h20191030599@hyderabad.bits-pilani.ac.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Errno 2] No such file or directory: '/home/paravasthu/ghostee/mailSender/test_cases/test_attachments/hema.jpg'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">replace() argument 2 must be str, not None</t>
   </si>
 </sst>
 </file>
@@ -116,7 +93,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -138,14 +115,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <vertAlign val="superscript"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -190,8 +159,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -212,50 +185,82 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="14.515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="14.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="37.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1020" style="0" width="11.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1020" style="1" width="11.52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="0" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="shashankp96@gmail.com"/>
-    <hyperlink ref="A3" r:id="rId2" display="h20191030599@hyderabad.bits-pilani.ac.in"/>
+    <hyperlink ref="A4" r:id="rId2" display="h20191030599@hyderabad.bits-pilani.ac.in"/>
+    <hyperlink ref="A5" r:id="rId3" display="hemapkrishna@gmail.com"/>
+    <hyperlink ref="A6" r:id="rId4" display="arkvidhatha@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555555" footer="0.511805555555555"/>
@@ -265,4 +270,66 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.06"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added exception handling in send_mails
</commit_message>
<xml_diff>
--- a/test_cases/RamaNamaCerti.xlsx
+++ b/test_cases/RamaNamaCerti.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t xml:space="preserve">emails</t>
   </si>
@@ -65,25 +65,16 @@
     <t xml:space="preserve">6th Feb 1993</t>
   </si>
   <si>
-    <t xml:space="preserve">arkvidhatha@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17th november 1997</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Errno 2] No such file or directory: '/home/paravasthu/ghostee/mailSender/test_cases/test_attachments/shashank.jpg'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{'shashank': (553, b'5.1.3 The recipient address &lt;shashank&gt; is not a valid RFC-5321 address. kf10sm2286206pjb.2 - gsmtp')}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sent mail to: h20191030599@hyderabad.bits-pilani.ac.in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Errno 2] No such file or directory: '/home/paravasthu/ghostee/mailSender/test_cases/test_attachments/hema.jpg'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">replace() argument 2 must be str, not None</t>
+    <t xml:space="preserve">sent mail from sheshu.emails@gmail.com to shashankp96@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{'shashank': (553, b'5.1.3 The recipient address &lt;shashank&gt; is not a valid RFC-5321 address. gd14sm2755376pjb.0 - gsmtp')}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sent mail from sheshu.emails@gmail.com to h20191030599@hyderabad.bits-pilani.ac.in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sent mail from sheshu.emails@gmail.com to hemapkrishna@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -185,8 +176,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="14.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="14.75" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1020" style="1" width="11.52"/>
@@ -247,20 +238,11 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" display="shashankp96@gmail.com"/>
     <hyperlink ref="A4" r:id="rId2" display="h20191030599@hyderabad.bits-pilani.ac.in"/>
     <hyperlink ref="A5" r:id="rId3" display="hemapkrishna@gmail.com"/>
-    <hyperlink ref="A6" r:id="rId4" display="arkvidhatha@gmail.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555555" footer="0.511805555555555"/>
@@ -277,50 +259,39 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.06"/>
-  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="0" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>